<commit_message>
correção de exibição de dados e atualização da base xlsx
</commit_message>
<xml_diff>
--- a/data/candidatos.xlsx
+++ b/data/candidatos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://senac144-my.sharepoint.com/personal/patrick_nascimento_pa_senac_br/Documents/CSEP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="41" documentId="13_ncr:1_{AD74628D-BE06-4FC1-BE04-2187DD70E9AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{92F89762-2E51-4862-AC5B-1527B237AAB1}"/>
+  <xr:revisionPtr revIDLastSave="47" documentId="13_ncr:1_{AD74628D-BE06-4FC1-BE04-2187DD70E9AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD5C6C0F-C3A3-4DA3-A561-D95190710020}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="128">
   <si>
     <t>Id</t>
   </si>
@@ -367,6 +367,60 @@
   </si>
   <si>
     <t>91981957348</t>
+  </si>
+  <si>
+    <t>Ana Clara Menezes Barroso</t>
+  </si>
+  <si>
+    <t>orquidea412016@gmail.com</t>
+  </si>
+  <si>
+    <t>91 982770312</t>
+  </si>
+  <si>
+    <t>Cursando no Senac  Desenvolvimento de Games 2026.</t>
+  </si>
+  <si>
+    <t>Professor Ivo Barbosa</t>
+  </si>
+  <si>
+    <t>Max Henrique da Cruz palha</t>
+  </si>
+  <si>
+    <t>maxhenrique12383@gmail.com</t>
+  </si>
+  <si>
+    <t>918596-8805</t>
+  </si>
+  <si>
+    <t>curso técnico de informática</t>
+  </si>
+  <si>
+    <t>Simone Amaral</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bento Monteiro do Couto </t>
+  </si>
+  <si>
+    <t>bentomonteiro10@gmail.com</t>
+  </si>
+  <si>
+    <t>91986284445</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Técnico de Informática </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Juan Gabriel Mendez dos Santos </t>
+  </si>
+  <si>
+    <t>juangabrielmendezdossantos@gmal.com</t>
+  </si>
+  <si>
+    <t>91981236651</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simone </t>
   </si>
 </sst>
 </file>
@@ -402,7 +456,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -412,13 +466,14 @@
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="9">
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -427,7 +482,7 @@
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -458,8 +513,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="OfficeForms.Table" displayName="OfficeForms.Table" ref="A1:L22" totalsRowShown="0">
-  <autoFilter ref="A1:L22" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="OfficeForms.Table" displayName="OfficeForms.Table" ref="A1:L27" totalsRowShown="0">
+  <autoFilter ref="A1:L27" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Id" dataDxfId="8">
       <extLst>
@@ -503,14 +558,14 @@
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Informe um email para contato" dataDxfId="1">
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Informe um email para contato" dataDxfId="4">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="rc7d435c89dda4bc4abd1199f19a527be"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Informe um número de contato" dataDxfId="0">
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Informe um número de contato" dataDxfId="3">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r387b0e56ae3742a3a30ecb64ca287eb4"/>
@@ -524,26 +579,26 @@
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Qual foi o último curso feito ou cursando no Senac?" dataDxfId="4">
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Qual foi o último curso feito ou cursando no Senac?" dataDxfId="2">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r568ac032fad94fd5ab2896b463a54e65"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Qual é o nome do instrutor que esteve ministrando as aula para você?" dataDxfId="3">
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Qual é o nome do instrutor que esteve ministrando as aula para você?" dataDxfId="1">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r9074ff20b62e4b0990664cefcf65c8b3"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{3C6772B8-4469-4D4C-BB84-00CF593C4E68}" name="CPF" dataDxfId="2"/>
+    <tableColumn id="12" xr3:uid="{3C6772B8-4469-4D4C-BB84-00CF593C4E68}" name="CPF" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
   <extLst>
     <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{839C7E11-91E4-4DBD-9C5D-0DEA604FA9AC}">
-      <xlmsforms:msForm id="EEV3fJkFaUCqMZJsRu0ZCaS-UizYaqVAixDVHdWZgvVUNjZNNTlTTjJZTkRBR1pRVVVFWlk0UFRGVi4u" isFormConnected="1" maxResponseId="21" latestEventMarker="10">
+      <xlmsforms:msForm id="EEV3fJkFaUCqMZJsRu0ZCaS-UizYaqVAixDVHdWZgvVUNjZNNTlTTjJZTkRBR1pRVVVFWlk0UFRGVi4u" isFormConnected="1" maxResponseId="26" latestEventMarker="15">
         <xlmsforms:syncedQuestionId>id</xlmsforms:syncedQuestionId>
         <xlmsforms:syncedQuestionId>startDate</xlmsforms:syncedQuestionId>
         <xlmsforms:syncedQuestionId>submitDate</xlmsforms:syncedQuestionId>
@@ -861,7 +916,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="20" hidden="1" customWidth="1"/>
@@ -1616,6 +1671,176 @@
       </c>
       <c r="L22" s="3"/>
     </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2">
+        <v>46182.509421296301</v>
+      </c>
+      <c r="C23" s="2">
+        <v>46182.522210648203</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="E23" s="3"/>
+      <c r="F23" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="H23" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="I23" s="1">
+        <v>38694</v>
+      </c>
+      <c r="J23" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="K23" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="L23" s="3"/>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2">
+        <v>46185.6860185185</v>
+      </c>
+      <c r="C24" s="2">
+        <v>46185.687743055598</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="E24" s="3"/>
+      <c r="F24" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="G24" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="H24" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="I24" s="1">
+        <v>39566</v>
+      </c>
+      <c r="J24" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="K24" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="L24" s="3"/>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2">
+        <v>46185.712094907401</v>
+      </c>
+      <c r="C25" s="2">
+        <v>46185.712812500002</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="E25" s="3"/>
+      <c r="F25" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="G25" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="H25" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="I25" s="1">
+        <v>39566</v>
+      </c>
+      <c r="J25" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="K25" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="L25" s="3"/>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2">
+        <v>46185.712500000001</v>
+      </c>
+      <c r="C26" s="2">
+        <v>46185.715543981503</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="E26" s="3"/>
+      <c r="F26" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="G26" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="H26" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="I26" s="1">
+        <v>39363</v>
+      </c>
+      <c r="J26" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="K26" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="L26" s="3"/>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A27" s="7">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2">
+        <v>46185.839097222197</v>
+      </c>
+      <c r="C27" s="2">
+        <v>46185.840381944399</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="E27" s="3"/>
+      <c r="F27" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="G27" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="H27" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="I27" s="1">
+        <v>39050</v>
+      </c>
+      <c r="J27" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="K27" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="L27" s="3"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="51" orientation="landscape" r:id="rId1"/>

</xml_diff>